<commit_message>
Tweaks to DCM input files.
</commit_message>
<xml_diff>
--- a/Inputs/DCM_template_parameters_Exposure.xlsx
+++ b/Inputs/DCM_template_parameters_Exposure.xlsx
@@ -2352,8 +2352,8 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="878a2fbfe6fee2aa092ffb79eb0579a1">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="376b02366c9bc1743b7b5079a857fb71" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
     <xsd:import namespace="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint.v3"/>
@@ -2887,7 +2887,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AE393AF-D13A-4280-965F-0527E409853E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51D577E9-3AC0-4243-84D1-EEEA024D6BC5}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>